<commit_message>
Fix figures and manuscript: remove EaP from year-by-year; 90% CI with t-quantiles; correct confounding explanation
</commit_message>
<xml_diff>
--- a/results/regression_output/full_sample_covid_analysis/extended_control_specifications.xlsx
+++ b/results/regression_output/full_sample_covid_analysis/extended_control_specifications.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:W9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,11 @@
           <t>r_squared</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>df_resid</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -560,28 +565,28 @@
         <v>-0.3586832490258667</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1258002088862993</v>
+        <v>0.1114079656052606</v>
       </c>
       <c r="J2" t="n">
-        <v>0.004563045486056572</v>
+        <v>0.001380347208086219</v>
       </c>
       <c r="K2" t="n">
         <v>0.1086117580486053</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1331184255773259</v>
+        <v>0.07195758655837421</v>
       </c>
       <c r="M2" t="n">
-        <v>0.41500303022429</v>
+        <v>0.1319278750416322</v>
       </c>
       <c r="N2" t="n">
         <v>0.06278039569190315</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1706963681708208</v>
+        <v>0.1179408932434768</v>
       </c>
       <c r="P2" t="n">
-        <v>0.713209218400954</v>
+        <v>0.5947879412813544</v>
       </c>
       <c r="Q2" t="n">
         <v>0.2994183188245934</v>
@@ -600,6 +605,9 @@
       </c>
       <c r="V2" t="n">
         <v>0.4222868362410958</v>
+      </c>
+      <c r="W2" t="n">
+        <v>434</v>
       </c>
     </row>
     <row r="3">
@@ -634,28 +642,28 @@
         <v>-0.3329291586321067</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1114265192535013</v>
+        <v>0.1167778909793696</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00296671404494453</v>
+        <v>0.004564214508270714</v>
       </c>
       <c r="K3" t="n">
         <v>0.0971936324649034</v>
       </c>
       <c r="L3" t="n">
-        <v>0.08260285374182259</v>
+        <v>0.05573016781682696</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2399777433067629</v>
+        <v>0.08185834096701994</v>
       </c>
       <c r="N3" t="n">
         <v>0.0245511174660307</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1370112169452358</v>
+        <v>0.1214375057206401</v>
       </c>
       <c r="P3" t="n">
-        <v>0.8578707430841943</v>
+        <v>0.839876855855858</v>
       </c>
       <c r="Q3" t="n">
         <v>0.2336543268663729</v>
@@ -674,6 +682,9 @@
       </c>
       <c r="V3" t="n">
         <v>0.3824041367382668</v>
+      </c>
+      <c r="W3" t="n">
+        <v>439</v>
       </c>
     </row>
     <row r="4">
@@ -708,28 +719,28 @@
         <v>-0.3504785606556576</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1187486325964152</v>
+        <v>0.1298652008380899</v>
       </c>
       <c r="J4" t="n">
-        <v>0.003331718724750354</v>
+        <v>0.007226513156255443</v>
       </c>
       <c r="K4" t="n">
         <v>0.09937366898180935</v>
       </c>
       <c r="L4" t="n">
-        <v>0.08999448954050022</v>
+        <v>0.05284827609630227</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2701000616232445</v>
+        <v>0.06071815597690922</v>
       </c>
       <c r="N4" t="n">
         <v>0.0108812817654662</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1451629858822026</v>
+        <v>0.1299954669441022</v>
       </c>
       <c r="P4" t="n">
-        <v>0.9402812715280882</v>
+        <v>0.9333288953422176</v>
       </c>
       <c r="Q4" t="n">
         <v>0.242609012380568</v>
@@ -748,6 +759,9 @@
       </c>
       <c r="V4" t="n">
         <v>0.379178849657785</v>
+      </c>
+      <c r="W4" t="n">
+        <v>441</v>
       </c>
     </row>
     <row r="5">
@@ -782,28 +796,28 @@
         <v>-0.3538577295275603</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1381615423428651</v>
+        <v>0.1361065710659744</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01076240081793411</v>
+        <v>0.009638456911854165</v>
       </c>
       <c r="K5" t="n">
         <v>0.155313073613081</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0982622259608591</v>
+        <v>0.07820403868661886</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1146853001705139</v>
+        <v>0.04765082758897754</v>
       </c>
       <c r="N5" t="n">
         <v>0.04370246834340927</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1695623367957826</v>
+        <v>0.1353140122663301</v>
       </c>
       <c r="P5" t="n">
-        <v>0.7967299313572329</v>
+        <v>0.7468701235207895</v>
       </c>
       <c r="Q5" t="n">
         <v>0.3146932641459779</v>
@@ -822,6 +836,9 @@
       </c>
       <c r="V5" t="n">
         <v>0.3384057745921305</v>
+      </c>
+      <c r="W5" t="n">
+        <v>442</v>
       </c>
     </row>
     <row r="6">
@@ -856,28 +873,28 @@
         <v>-0.3417128272472357</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1539856791575077</v>
+        <v>0.1309100979924854</v>
       </c>
       <c r="J6" t="n">
-        <v>0.02698671061535518</v>
+        <v>0.009354603047433407</v>
       </c>
       <c r="K6" t="n">
         <v>0.1576019215748242</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1026977164102668</v>
+        <v>0.08081523800364121</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1255943976835276</v>
+        <v>0.05179133588135487</v>
       </c>
       <c r="N6" t="n">
         <v>0.05443345894513896</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1811982683528159</v>
+        <v>0.1321989119521975</v>
       </c>
       <c r="P6" t="n">
-        <v>0.7640073163452419</v>
+        <v>0.6807196342300188</v>
       </c>
       <c r="Q6" t="n">
         <v>0.3145453332248944</v>
@@ -896,6 +913,9 @@
       </c>
       <c r="V6" t="n">
         <v>0.3381409205256601</v>
+      </c>
+      <c r="W6" t="n">
+        <v>441</v>
       </c>
     </row>
     <row r="7">
@@ -930,28 +950,28 @@
         <v>-0.4183164000911773</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1187380505751605</v>
+        <v>0.1210348275559162</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0004712910068762621</v>
+        <v>0.0006011351914416707</v>
       </c>
       <c r="K7" t="n">
         <v>0.1762019955230177</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1321795283334539</v>
+        <v>0.07348566307227336</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1832050097293021</v>
+        <v>0.01691086741580072</v>
       </c>
       <c r="N7" t="n">
         <v>0.01785109638434906</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1692039517198653</v>
+        <v>0.1216546957945579</v>
       </c>
       <c r="P7" t="n">
-        <v>0.9160267753934808</v>
+        <v>0.8834077847480817</v>
       </c>
       <c r="Q7" t="n">
         <v>0.3315563110139996</v>
@@ -970,6 +990,9 @@
       </c>
       <c r="V7" t="n">
         <v>0.3768682934293673</v>
+      </c>
+      <c r="W7" t="n">
+        <v>440</v>
       </c>
     </row>
     <row r="8">
@@ -1004,28 +1027,28 @@
         <v>-0.3506577463163462</v>
       </c>
       <c r="I8" t="n">
-        <v>0.142932098770189</v>
+        <v>0.1342793207607255</v>
       </c>
       <c r="J8" t="n">
-        <v>0.01454059203119495</v>
+        <v>0.009324514578489707</v>
       </c>
       <c r="K8" t="n">
         <v>0.1442811853744973</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1094396141579807</v>
+        <v>0.07370603774560643</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1880663167692185</v>
+        <v>0.0509164389700778</v>
       </c>
       <c r="N8" t="n">
         <v>0.05126825892725741</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1760570296726802</v>
+        <v>0.1278369863875255</v>
       </c>
       <c r="P8" t="n">
-        <v>0.7710333112954051</v>
+        <v>0.6885819546299945</v>
       </c>
       <c r="Q8" t="n">
         <v>0.3295705458221864</v>
@@ -1044,6 +1067,9 @@
       </c>
       <c r="V8" t="n">
         <v>0.3449049784719663</v>
+      </c>
+      <c r="W8" t="n">
+        <v>441</v>
       </c>
     </row>
     <row r="9">
@@ -1078,28 +1104,28 @@
         <v>-0.3498175481283099</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1471080883824976</v>
+        <v>0.1373276326968269</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01783189491473158</v>
+        <v>0.01119232494960265</v>
       </c>
       <c r="K9" t="n">
         <v>0.1540962292337341</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1049409266491931</v>
+        <v>0.07629162331292183</v>
       </c>
       <c r="M9" t="n">
-        <v>0.142702765369304</v>
+        <v>0.04400236755850839</v>
       </c>
       <c r="N9" t="n">
         <v>0.04806953732053527</v>
       </c>
       <c r="O9" t="n">
-        <v>0.1777773313817092</v>
+        <v>0.1373934621959423</v>
       </c>
       <c r="P9" t="n">
-        <v>0.7869847517457584</v>
+        <v>0.7266042441438947</v>
       </c>
       <c r="Q9" t="n">
         <v>0.3217204946260342</v>
@@ -1118,6 +1144,9 @@
       </c>
       <c r="V9" t="n">
         <v>0.3365123578311333</v>
+      </c>
+      <c r="W9" t="n">
+        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>